<commit_message>
actualiza acumulados 17/06/2026 15:34
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
@@ -819,7 +819,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6618,7 +6618,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9112,7 +9112,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9618,7 +9618,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9871,7 +9871,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -10124,7 +10124,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10377,7 +10377,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10883,7 +10883,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -11136,7 +11136,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11389,7 +11389,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11642,7 +11642,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -12148,7 +12148,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -12401,7 +12401,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -12654,7 +12654,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -13160,7 +13160,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -14425,7 +14425,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -14678,7 +14678,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -14931,7 +14931,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -15437,7 +15437,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -15939,7 +15939,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -16192,7 +16192,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -16445,7 +16445,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -16951,7 +16951,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -17204,7 +17204,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -17457,7 +17457,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -17710,7 +17710,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -17963,7 +17963,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -18212,7 +18212,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -18465,7 +18465,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -18718,7 +18718,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -19224,7 +19224,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -19477,7 +19477,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -19730,7 +19730,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -19979,7 +19979,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -20232,7 +20232,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -20485,7 +20485,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -21240,7 +21240,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -21493,7 +21493,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -21746,7 +21746,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -21999,7 +21999,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -22252,7 +22252,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESTRELLITA (IED)</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">

</xml_diff>

<commit_message>
actualiza acumulados 19/06/2026 14:49
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
@@ -858,9 +858,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -1360,9 +1360,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1613,9 +1613,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -2372,9 +2372,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -2878,9 +2878,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -3882,9 +3882,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -4380,9 +4380,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -4886,9 +4886,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -5392,9 +5392,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -5645,9 +5645,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -5898,9 +5898,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -7633,9 +7633,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -8139,9 +8139,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -8392,9 +8392,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -9151,9 +9151,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr">
-        <is>
-          <t>CORRECTO</t>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -9404,9 +9404,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -10669,9 +10669,9 @@
           <t>D</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>INCORRECTO</t>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>CORRECTO</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">

</xml_diff>

<commit_message>
actualiza acumulados 25/06/2026 10:51
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COL. ESTRELLITA 702_CALIFICADO.xlsx
@@ -807,11 +807,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -819,7 +815,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1060,11 +1056,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -1072,7 +1064,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1309,11 +1301,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -1321,7 +1309,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1562,11 +1550,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -1574,7 +1558,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1815,11 +1799,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -1827,7 +1807,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2068,11 +2048,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -2080,7 +2056,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2321,11 +2297,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -2333,7 +2305,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2574,11 +2546,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -2586,7 +2554,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2827,11 +2795,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -2839,7 +2803,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3072,11 +3036,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -3084,7 +3044,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3325,11 +3285,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -3337,7 +3293,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3578,11 +3534,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="inlineStr"/>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -3590,7 +3542,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3831,11 +3783,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -3843,7 +3791,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4084,11 +4032,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -4096,7 +4040,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4329,11 +4273,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -4341,7 +4281,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4582,11 +4522,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -4594,7 +4530,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4835,11 +4771,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="inlineStr"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -4847,7 +4779,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5088,11 +5020,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
       <c r="B19" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -5100,7 +5028,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5341,11 +5269,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
       <c r="B20" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -5353,7 +5277,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -5594,11 +5518,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -5606,7 +5526,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5847,11 +5767,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
       <c r="B22" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -5859,7 +5775,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -6100,11 +6016,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
       <c r="B23" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -6112,7 +6024,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6353,11 +6265,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="inlineStr"/>
       <c r="B24" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -6365,7 +6273,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6606,11 +6514,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="inlineStr"/>
       <c r="B25" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -6618,7 +6522,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -6859,11 +6763,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="inlineStr"/>
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -6871,7 +6771,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -7088,11 +6988,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -7100,7 +6996,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7341,11 +7237,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr"/>
       <c r="B28" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -7353,7 +7245,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -7582,11 +7474,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -7594,7 +7482,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7835,11 +7723,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -7847,7 +7731,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -8088,11 +7972,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -8100,7 +7980,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8341,11 +8221,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -8353,7 +8229,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -8594,11 +8470,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="inlineStr"/>
       <c r="B33" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -8606,7 +8478,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -8847,11 +8719,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="inlineStr"/>
       <c r="B34" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -8859,7 +8727,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9100,11 +8968,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
       <c r="B35" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -9112,7 +8976,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9353,11 +9217,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
       <c r="B36" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -9365,7 +9225,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9606,11 +9466,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
       <c r="B37" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -9618,7 +9474,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9859,11 +9715,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -9871,7 +9723,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -10112,11 +9964,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr"/>
       <c r="B39" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -10124,7 +9972,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10365,11 +10213,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="inlineStr"/>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -10377,7 +10221,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10618,11 +10462,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="inlineStr"/>
       <c r="B41" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -10630,7 +10470,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10871,11 +10711,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A42" s="2" t="inlineStr"/>
       <c r="B42" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -10883,7 +10719,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -11124,11 +10960,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="inlineStr"/>
       <c r="B43" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -11136,7 +10968,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11377,11 +11209,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -11389,7 +11217,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11630,11 +11458,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -11642,7 +11466,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11883,11 +11707,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -11895,7 +11715,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -12136,11 +11956,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="inlineStr"/>
       <c r="B47" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -12148,7 +11964,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -12389,11 +12205,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -12401,7 +12213,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -12642,11 +12454,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="inlineStr"/>
       <c r="B49" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -12654,7 +12462,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -12895,11 +12703,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -12907,7 +12711,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -13148,11 +12952,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A51" s="2" t="inlineStr"/>
       <c r="B51" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -13160,7 +12960,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -13401,11 +13201,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -13413,7 +13209,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13654,11 +13450,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A53" s="2" t="inlineStr"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -13666,7 +13458,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -13907,11 +13699,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="inlineStr"/>
       <c r="B54" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -13919,7 +13707,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -14160,11 +13948,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A55" s="2" t="inlineStr"/>
       <c r="B55" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -14172,7 +13956,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -14413,11 +14197,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A56" s="2" t="inlineStr"/>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -14425,7 +14205,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -14666,11 +14446,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A57" s="2" t="inlineStr"/>
       <c r="B57" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -14678,7 +14454,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -14919,11 +14695,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A58" s="2" t="inlineStr"/>
       <c r="B58" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -14931,7 +14703,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -15172,11 +14944,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="inlineStr"/>
       <c r="B59" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -15184,7 +14952,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -15425,11 +15193,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A60" s="2" t="inlineStr"/>
       <c r="B60" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -15437,7 +15201,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -15678,11 +15442,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A61" s="2" t="inlineStr"/>
       <c r="B61" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -15690,7 +15450,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -15927,11 +15687,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A62" s="2" t="inlineStr"/>
       <c r="B62" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -15939,7 +15695,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -16180,11 +15936,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A63" s="2" t="inlineStr"/>
       <c r="B63" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -16192,7 +15944,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -16433,11 +16185,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A64" s="2" t="inlineStr"/>
       <c r="B64" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -16445,7 +16193,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -16686,11 +16434,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A65" s="2" t="inlineStr"/>
       <c r="B65" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -16698,7 +16442,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -16939,11 +16683,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A66" s="2" t="inlineStr"/>
       <c r="B66" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -16951,7 +16691,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -17192,11 +16932,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A67" s="2" t="inlineStr"/>
       <c r="B67" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -17204,7 +16940,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -17445,11 +17181,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A68" s="2" t="inlineStr"/>
       <c r="B68" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -17457,7 +17189,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -17698,11 +17430,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A69" s="2" t="inlineStr"/>
       <c r="B69" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -17710,7 +17438,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -17951,11 +17679,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A70" s="2" t="inlineStr"/>
       <c r="B70" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -17963,7 +17687,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -18200,11 +17924,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A71" s="2" t="inlineStr"/>
       <c r="B71" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -18212,7 +17932,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -18453,11 +18173,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A72" s="2" t="inlineStr"/>
       <c r="B72" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -18465,7 +18181,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -18706,11 +18422,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A73" s="2" t="inlineStr"/>
       <c r="B73" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -18718,7 +18430,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -18959,11 +18671,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A74" s="2" t="inlineStr"/>
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -18971,7 +18679,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -19212,11 +18920,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A75" s="2" t="inlineStr"/>
       <c r="B75" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -19224,7 +18928,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -19465,11 +19169,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A76" s="2" t="inlineStr"/>
       <c r="B76" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -19477,7 +19177,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -19718,11 +19418,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A77" s="2" t="inlineStr"/>
       <c r="B77" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -19730,7 +19426,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -19967,11 +19663,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A78" s="2" t="inlineStr"/>
       <c r="B78" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -19979,7 +19671,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -20220,11 +19912,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A79" s="2" t="inlineStr"/>
       <c r="B79" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -20232,7 +19920,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -20473,11 +20161,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A80" s="2" t="inlineStr"/>
       <c r="B80" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -20485,7 +20169,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -20726,11 +20410,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A81" s="2" t="inlineStr"/>
       <c r="B81" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -20738,7 +20418,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -20979,11 +20659,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A82" s="2" t="inlineStr"/>
       <c r="B82" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -20991,7 +20667,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -21228,11 +20904,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A83" s="2" t="inlineStr"/>
       <c r="B83" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -21240,7 +20912,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -21481,11 +21153,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A84" s="2" t="inlineStr"/>
       <c r="B84" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -21493,7 +21161,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -21734,11 +21402,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A85" s="2" t="inlineStr"/>
       <c r="B85" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -21746,7 +21410,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -21987,11 +21651,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A86" s="2" t="inlineStr"/>
       <c r="B86" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -21999,7 +21659,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -22240,11 +21900,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>TRATADO</t>
-        </is>
-      </c>
+      <c r="A87" s="2" t="inlineStr"/>
       <c r="B87" s="2" t="inlineStr">
         <is>
           <t>111001098612</t>
@@ -22252,7 +21908,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESTRELLITA (IED)</t>
+          <t>COLEGIO LA ESTRELLITA (IED) - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">

</xml_diff>